<commit_message>
adding lab 2 stuff
</commit_message>
<xml_diff>
--- a/docs/project/Lab_01_rubric.xlsx
+++ b/docs/project/Lab_01_rubric.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{3A943D7E-B3DD-D74C-9A1F-CB635474BF2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="30680" windowHeight="27900" xr2:uid="{667F11EA-4EF5-B244-B65C-9CA4E22D96EF}"/>
+    <workbookView xWindow="22980" yWindow="600" windowWidth="30680" windowHeight="27900" xr2:uid="{667F11EA-4EF5-B244-B65C-9CA4E22D96EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>